<commit_message>
Added values of the sale Acordo, Acordo Judicial and CMI
</commit_message>
<xml_diff>
--- a/data/Custo Receita 2025 Int.xlsx
+++ b/data/Custo Receita 2025 Int.xlsx
@@ -4893,7 +4893,7 @@
         <v/>
       </c>
       <c r="M7" s="263" t="n">
-        <v>179798.76</v>
+        <v>1</v>
       </c>
       <c r="N7" s="261">
         <f>M7-L7</f>
@@ -4958,7 +4958,7 @@
         <v/>
       </c>
       <c r="M9" s="263" t="n">
-        <v>33545</v>
+        <v>13</v>
       </c>
       <c r="N9" s="261">
         <f>M9-L9</f>
@@ -6093,7 +6093,7 @@
         <v/>
       </c>
       <c r="M40" s="263" t="n">
-        <v>36515</v>
+        <v>14</v>
       </c>
       <c r="N40" s="261">
         <f>M40-L40</f>
@@ -7248,7 +7248,7 @@
         <v/>
       </c>
       <c r="M71" s="263" t="n">
-        <v>37165</v>
+        <v>15</v>
       </c>
       <c r="N71" s="261">
         <f>M71-L71</f>
@@ -8402,7 +8402,7 @@
         <v/>
       </c>
       <c r="M102" s="263" t="n">
-        <v>38805</v>
+        <v>16</v>
       </c>
       <c r="N102" s="261">
         <f>M102-L102</f>
@@ -9475,7 +9475,7 @@
         <v/>
       </c>
       <c r="M131" s="263" t="n">
-        <v>174759.02</v>
+        <v>5</v>
       </c>
       <c r="N131" s="261">
         <f>M131-L131</f>
@@ -9540,7 +9540,7 @@
         <v/>
       </c>
       <c r="M133" s="263" t="n">
-        <v>37635</v>
+        <v>17</v>
       </c>
       <c r="N133" s="261">
         <f>M133-L133</f>
@@ -10621,7 +10621,7 @@
         <v/>
       </c>
       <c r="M162" s="263" t="n">
-        <v>14466.76</v>
+        <v>6</v>
       </c>
       <c r="N162" s="261">
         <f>M162-L162</f>
@@ -10686,7 +10686,7 @@
         <v/>
       </c>
       <c r="M164" s="263" t="n">
-        <v>40635</v>
+        <v>18</v>
       </c>
       <c r="N164" s="261">
         <f>M164-L164</f>

</xml_diff>